<commit_message>
feat(items): add material group code column to the directs excel import
</commit_message>
<xml_diff>
--- a/src/api/items/templates/items-import-template.xlsx
+++ b/src/api/items/templates/items-import-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>Mã vật tư</t>
   </si>
@@ -32,6 +32,9 @@
     <t>Mã khách hàng</t>
   </si>
   <si>
+    <t>Mã nhóm vật tư</t>
+  </si>
+  <si>
     <t>Định mức tồn tối thiểu</t>
   </si>
   <si>
@@ -98,7 +101,7 @@
     <t>Cột tiêu đề màu đỏ là bắt buộc: Mã vật tư, Tên vật tư, Mã đơn vị tính.</t>
   </si>
   <si>
-    <t>Mã đơn vị tính / Mã nhà cung cấp / Mã khách hàng phải là mã đã có trong hệ thống (không dùng tên).</t>
+    <t>Mã đơn vị tính / Mã nhà cung cấp / Mã khách hàng / Mã nhóm vật tư phải là mã đã có trong hệ thống (không dùng tên).</t>
   </si>
   <si>
     <t>Phiên bản bỏ trống = R01. Mã vật tư + phiên bản không được trùng vật tư đã có hoặc trùng giữa các dòng.</t>
@@ -490,22 +493,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="21" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="13" width="18" customWidth="1"/>
-    <col min="14" max="14" width="23" customWidth="1"/>
-    <col min="15" max="16" width="18" customWidth="1"/>
+    <col min="6" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="23" customWidth="1"/>
+    <col min="12" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="23" customWidth="1"/>
+    <col min="16" max="17" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -554,34 +557,34 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2">
+        <v>21</v>
+      </c>
+      <c r="H2">
         <v>100</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>7.85</v>
-      </c>
-      <c r="I2" t="s">
-        <v>21</v>
       </c>
       <c r="J2" t="s">
         <v>22</v>
@@ -590,24 +593,27 @@
         <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="M2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N2" t="s">
         <v>25</v>
       </c>
       <c r="O2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="P2" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -621,31 +627,31 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>